<commit_message>
Completion of python phase one
</commit_message>
<xml_diff>
--- a/Python/Python.xlsx
+++ b/Python/Python.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Learner\Recap\Python\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66FC23B3-75B6-4022-9831-E19EFE63B73A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B7DBB3A-6BDC-4E96-A739-BB5CAB2B46B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -142,42 +142,14 @@
     <t>Using the typing module (List, Dict, Optional); heavily used in FastAPI.</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Reference counting,</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="7"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> the garbage collector</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, and memory leaks.</t>
-    </r>
+    <t>Reference counting, the garbage collector, and memory leaks.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -204,22 +176,8 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="10"/>
-      <color theme="7"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="6">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -234,19 +192,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -263,21 +209,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -517,13 +458,13 @@
       <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
+      <c r="I1" s="8"/>
     </row>
     <row r="2" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
@@ -538,67 +479,67 @@
       <c r="D2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
-      <c r="I2" s="5"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="7"/>
     </row>
     <row r="3" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" s="13" t="s">
+      <c r="C3" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="F3" s="12"/>
-      <c r="G3" s="12"/>
-      <c r="H3" s="12"/>
-      <c r="I3" s="12"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
     </row>
     <row r="4" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="D4" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="E4" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
-      <c r="H4" s="10"/>
-      <c r="I4" s="10"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
+      <c r="I4" s="6"/>
     </row>
     <row r="5" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="3" t="s">
         <v>8</v>
       </c>
       <c r="E5" s="7" t="s">
@@ -610,16 +551,16 @@
       <c r="I5" s="7"/>
     </row>
     <row r="6" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6" s="4" t="s">
+      <c r="C6" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="3" t="s">
         <v>11</v>
       </c>
       <c r="E6" s="7" t="s">
@@ -631,37 +572,37 @@
       <c r="I6" s="7"/>
     </row>
     <row r="7" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="9" t="s">
+      <c r="A7" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" s="10" t="s">
+      <c r="C7" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F7" s="10"/>
-      <c r="G7" s="10"/>
-      <c r="H7" s="10"/>
-      <c r="I7" s="10"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
     </row>
     <row r="8" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="3" t="s">
         <v>22</v>
       </c>
       <c r="E8" s="7" t="s">
@@ -673,16 +614,16 @@
       <c r="I8" s="7"/>
     </row>
     <row r="9" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D9" s="4" t="s">
+      <c r="C9" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" s="3" t="s">
         <v>11</v>
       </c>
       <c r="E9" s="7" t="s">
@@ -694,88 +635,88 @@
       <c r="I9" s="7"/>
     </row>
     <row r="10" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+      <c r="A10" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="C10" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D10" s="1" t="s">
+      <c r="C10" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="E10" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
-      <c r="H10" s="8"/>
-      <c r="I10" s="8"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="6"/>
     </row>
     <row r="11" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+      <c r="A11" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="D11" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="E11" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
-      <c r="H11" s="8"/>
-      <c r="I11" s="8"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6"/>
+      <c r="H11" s="6"/>
+      <c r="I11" s="6"/>
     </row>
     <row r="12" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C12" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E12" s="5" t="s">
+      <c r="C12" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="5"/>
-      <c r="I12" s="5"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="6"/>
+      <c r="H12" s="6"/>
+      <c r="I12" s="6"/>
     </row>
     <row r="13" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
+      <c r="A13" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C13" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D13" s="1" t="s">
+      <c r="C13" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D13" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="E13" s="8" t="s">
+      <c r="E13" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
-      <c r="H13" s="8"/>
-      <c r="I13" s="8"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="7"/>
+      <c r="H13" s="7"/>
+      <c r="I13" s="7"/>
     </row>
     <row r="14" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
@@ -790,16 +731,21 @@
       <c r="D14" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="E14" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="F14" s="8"/>
-      <c r="G14" s="8"/>
-      <c r="H14" s="8"/>
-      <c r="I14" s="8"/>
+      <c r="F14" s="5"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="5"/>
+      <c r="I14" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="E2:I2"/>
+    <mergeCell ref="E1:I1"/>
+    <mergeCell ref="E3:I3"/>
+    <mergeCell ref="E5:I5"/>
+    <mergeCell ref="E6:I6"/>
     <mergeCell ref="E14:I14"/>
     <mergeCell ref="E4:I4"/>
     <mergeCell ref="E8:I8"/>
@@ -809,11 +755,6 @@
     <mergeCell ref="E12:I12"/>
     <mergeCell ref="E13:I13"/>
     <mergeCell ref="E7:I7"/>
-    <mergeCell ref="E2:I2"/>
-    <mergeCell ref="E1:I1"/>
-    <mergeCell ref="E3:I3"/>
-    <mergeCell ref="E5:I5"/>
-    <mergeCell ref="E6:I6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>